<commit_message>
Added Variables to API Key and other values that were hardcoded
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lap10\Downloads\Auxis-ReFramework_Windows-master (1)\Asana Project\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lap10\Documents\UiPath\Asana\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAAA85D4-EDFF-446A-A1EC-0EE4B752F08B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C45A944B-449B-4EAD-92AA-3B9CF88A046E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="89">
   <si>
     <t>Name</t>
   </si>
@@ -251,15 +251,9 @@
     <t>Adjunct Faculty Reappointment</t>
   </si>
   <si>
-    <t>Asana API</t>
-  </si>
-  <si>
     <t>AdjReappProjectID</t>
   </si>
   <si>
-    <t>ASANA_API</t>
-  </si>
-  <si>
     <t>Project ID Asana</t>
   </si>
   <si>
@@ -278,14 +272,32 @@
     <t>AdjunctReappointmentProcessTransactionQueue</t>
   </si>
   <si>
-    <t>C:\Users\lap10\Downloads\Auxis-ReFramework_Windows-master (1)\Asana Project\Data\Temp</t>
+    <t>ChairAdministrative</t>
+  </si>
+  <si>
+    <t>C. Fred Higgs</t>
+  </si>
+  <si>
+    <t>ASANA_API_V2</t>
+  </si>
+  <si>
+    <t>Faculty Administrative Specialist</t>
+  </si>
+  <si>
+    <t>AsanaAPI</t>
+  </si>
+  <si>
+    <t>AdministrativeSpecialist</t>
+  </si>
+  <si>
+    <t>Data\Temp</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -324,6 +336,12 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -345,7 +363,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -360,6 +378,7 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -702,7 +721,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z1004"/>
+  <dimension ref="A1:Z1005"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="43.5703125" customWidth="1"/>
@@ -808,7 +827,7 @@
         <v>73</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>21</v>
@@ -819,7 +838,7 @@
         <v>56</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>57</v>
@@ -849,143 +868,150 @@
     </row>
     <row r="8" spans="1:26" ht="15" customHeight="1">
       <c r="A8" t="s">
-        <v>80</v>
-      </c>
-      <c r="B8" t="s">
-        <v>84</v>
+        <v>78</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>88</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
-    <row r="9" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="10" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A10" s="6" t="s">
+    <row r="9" spans="1:26" ht="15" customHeight="1">
+      <c r="A9" t="s">
+        <v>82</v>
+      </c>
+      <c r="B9" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="10" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="11" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A11" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="B10" s="2"/>
-      <c r="C10" s="4"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="4"/>
     </row>
-    <row r="11" spans="1:26" ht="30">
-      <c r="A11" t="s">
+    <row r="12" spans="1:26" ht="30">
+      <c r="A12" t="s">
         <v>29</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B12" t="s">
         <v>38</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C12" s="3" t="s">
         <v>39</v>
-      </c>
-    </row>
-    <row r="12" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A12" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B12" s="2">
-        <v>30</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1">
       <c r="A13" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>35</v>
+        <v>30</v>
+      </c>
+      <c r="B13" s="2">
+        <v>30</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1">
       <c r="A14" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
       <c r="A15" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="B15" t="s">
-        <v>37</v>
-      </c>
-      <c r="C15" s="2"/>
+        <v>33</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1">
       <c r="A16" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>53</v>
-      </c>
+        <v>34</v>
+      </c>
+      <c r="B16" t="s">
+        <v>37</v>
+      </c>
+      <c r="C16" s="2"/>
     </row>
     <row r="17" spans="1:3" ht="14.25" customHeight="1">
       <c r="A17" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="B17" t="b">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="14.25" customHeight="1">
       <c r="A18" s="2" t="s">
-        <v>72</v>
+        <v>51</v>
       </c>
       <c r="B18" t="b">
         <v>0</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C18" s="4" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="14.25" customHeight="1">
       <c r="A19" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B19" t="b">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A20" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B19" t="s">
-        <v>82</v>
+      <c r="B20" t="s">
+        <v>80</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="21" spans="1:3" ht="15" customHeight="1">
-      <c r="A21" s="6" t="s">
+    <row r="21" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="22" spans="1:3" ht="15" customHeight="1">
+      <c r="A22" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="C21"/>
+      <c r="C22"/>
     </row>
-    <row r="22" spans="1:3" ht="15" customHeight="1">
-      <c r="A22" t="s">
+    <row r="23" spans="1:3" ht="15" customHeight="1">
+      <c r="A23" t="s">
         <v>40</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C23" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="12.75" customHeight="1">
-      <c r="A23" t="s">
+    <row r="24" spans="1:3" ht="12.75" customHeight="1">
+      <c r="A24" t="s">
         <v>44</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="C24" s="3" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="14.25" customHeight="1">
-      <c r="B24">
+    <row r="25" spans="1:3" ht="14.25" customHeight="1">
+      <c r="B25">
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="26" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A26" s="6" t="s">
+    <row r="26" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="27" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A27" s="6" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="28" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="29" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="30" spans="1:3" ht="14.25" customHeight="1"/>
@@ -1963,6 +1989,7 @@
     <row r="1002" ht="14.25" customHeight="1"/>
     <row r="1003" ht="14.25" customHeight="1"/>
     <row r="1004" ht="14.25" customHeight="1"/>
+    <row r="1005" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3153,7 +3180,7 @@
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="31.85546875" customWidth="1"/>
-    <col min="2" max="2" width="30.140625" customWidth="1"/>
+    <col min="2" max="2" width="50.85546875" customWidth="1"/>
     <col min="3" max="3" width="60.28515625" customWidth="1"/>
     <col min="4" max="26" width="65.42578125" customWidth="1"/>
   </cols>
@@ -3195,28 +3222,38 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A2" t="s">
-        <v>75</v>
+      <c r="A2" s="2" t="s">
+        <v>86</v>
       </c>
       <c r="B2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C2" t="s">
         <v>77</v>
-      </c>
-      <c r="C2" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="3" spans="1:26" ht="14.25" customHeight="1">
       <c r="A3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B3" t="s">
         <v>76</v>
       </c>
-      <c r="B3" t="s">
-        <v>78</v>
-      </c>
       <c r="C3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
-    <row r="4" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="4" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A4" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="C4" t="s">
+        <v>77</v>
+      </c>
+    </row>
     <row r="5" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="6" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="7" spans="1:26" ht="14.25" customHeight="1"/>
@@ -4214,5 +4251,6 @@
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added Logs in the code
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lap10\Documents\UiPath\Asana\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C45A944B-449B-4EAD-92AA-3B9CF88A046E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E09CC915-74A7-4E3A-9F09-B543232A424E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -275,9 +275,6 @@
     <t>ChairAdministrative</t>
   </si>
   <si>
-    <t>C. Fred Higgs</t>
-  </si>
-  <si>
     <t>ASANA_API_V2</t>
   </si>
   <si>
@@ -291,6 +288,9 @@
   </si>
   <si>
     <t>Data\Temp</t>
+  </si>
+  <si>
+    <t>C. Fred Higgs III</t>
   </si>
 </sst>
 </file>
@@ -871,7 +871,7 @@
         <v>78</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>79</v>
@@ -882,7 +882,7 @@
         <v>82</v>
       </c>
       <c r="B9" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1"/>
@@ -3223,10 +3223,10 @@
     </row>
     <row r="2" spans="1:26" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C2" t="s">
         <v>77</v>
@@ -3245,10 +3245,10 @@
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C4" t="s">
         <v>77</v>

</xml_diff>

<commit_message>
Added Logic after UAT
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lap10\Documents\UiPath\Asana\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57FA761F-AB4F-4B07-A877-B1402F8BAE49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C8896A3-389C-42F9-9874-26FE0827B0AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -275,9 +275,6 @@
     <t>ChairAdministrative</t>
   </si>
   <si>
-    <t>ASANA_API_V2</t>
-  </si>
-  <si>
     <t>Faculty Administrative Specialist</t>
   </si>
   <si>
@@ -291,6 +288,9 @@
   </si>
   <si>
     <t>C. Fred Higgs III</t>
+  </si>
+  <si>
+    <t>ASANA_API</t>
   </si>
 </sst>
 </file>
@@ -871,7 +871,7 @@
         <v>78</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>79</v>
@@ -882,7 +882,7 @@
         <v>82</v>
       </c>
       <c r="B9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1"/>
@@ -3223,10 +3223,10 @@
     </row>
     <row r="2" spans="1:26" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B2" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="C2" t="s">
         <v>77</v>
@@ -3245,10 +3245,10 @@
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C4" t="s">
         <v>77</v>

</xml_diff>